<commit_message>
Refresh Shiny app data 2026-09-21 19:52
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{020DC9AF-3FDB-4907-88FB-D57EC864C02C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A69E1680-BAA9-4EEF-B793-AE37DC0081BB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87AE9994-0DD6-451F-AADD-B5E5198EFF1E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841F6E23-6243-40A6-9108-ADB9E57FD55E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADA2A5DB-9E56-4289-B901-794D26DB6745}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDDAB82F-1911-4B54-AB0A-F30BD1DAD1FA}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-22 11:55
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -594,291 +594,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3dd70bd28c77d4108edb5ca6812bb84f">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cd59d6f2988212fc297a6d404d3fed4" ns2:_="" ns3:_="">
-    <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="12" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="16" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2a91012f-191a-4297-80da-223551dc3c4f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="25" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="17" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="18" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{ec99e049-fb75-4c8f-a4b4-b132771b9bd6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A69E1680-BAA9-4EEF-B793-AE37DC0081BB}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841F6E23-6243-40A6-9108-ADB9E57FD55E}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDDAB82F-1911-4B54-AB0A-F30BD1DAD1FA}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-23 11:02
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -594,291 +594,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3dd70bd28c77d4108edb5ca6812bb84f">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cd59d6f2988212fc297a6d404d3fed4" ns2:_="" ns3:_="">
-    <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="12" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="16" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2a91012f-191a-4297-80da-223551dc3c4f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="25" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="17" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="18" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{ec99e049-fb75-4c8f-a4b4-b132771b9bd6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6DEDBF0-FB5B-4ABF-B02A-76E8B8331B32}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58CD49DB-849B-4036-BF8A-13A4A55DBE95}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A3E71DA1-ECDA-4AAE-A35D-EF28D1B0A320}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-25 17:04
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32221B79-914F-40F6-8D44-7D0E3B00918F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F635FD6E-C41B-4F1B-B1A6-A3F554A93541}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{435D6D22-CFEA-4562-8493-5A505539B6BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDEB95E2-FCB5-49BB-B630-5CDA21BCBB59}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0029772-43D2-4667-AFCC-9F41E83C518C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8E8078E-B096-45BD-86CB-8ADA6D6FEDA2}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-26 00:15
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F635FD6E-C41B-4F1B-B1A6-A3F554A93541}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F2A4334-5534-4B28-BA80-00A5A9AF2D67}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDEB95E2-FCB5-49BB-B630-5CDA21BCBB59}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F2E171A-0099-41A4-B36E-8F3B5A128AB7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8E8078E-B096-45BD-86CB-8ADA6D6FEDA2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41555D2C-D078-45A4-A6FD-35BEA719A578}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-26 22:35
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F2A4334-5534-4B28-BA80-00A5A9AF2D67}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C79AE996-DF96-42E3-8631-C1D99AAE0E20}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F2E171A-0099-41A4-B36E-8F3B5A128AB7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{724323CF-A89C-49AE-835C-3F9B672CAA29}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41555D2C-D078-45A4-A6FD-35BEA719A578}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E926F03-D38A-4147-B226-7E335B90B3BE}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-27 14:01
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DBE1859-3690-4CB2-9FE5-CCF9ECA6DD53}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D73372BB-2B6B-4D08-87B3-0AF0F3FF42FE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD038A73-B6B6-4434-BBB7-AFE8829ACC8C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB3D38D5-AFCD-47A4-8605-E0272DF5E21D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{912665B3-83CD-4DC1-A98A-116C3B319AA0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FAE26D7E-C89B-407D-B0CD-29F87B623D67}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-29 01:20
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708FBBB3-68E4-48AC-B65A-5E0C859E1DA5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA933C46-8D80-48A1-943D-6FF7CBCBDD2F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{672697BE-2FAD-47CD-81D7-46B8A0C89737}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B3CC3FA-B2EA-4EA2-82F7-4F16E6897E69}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B768A1E1-A362-409A-971D-23225CB78C5F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A0BC28A-337D-469B-9D7B-B2ED6855629D}"/>
 </file>
</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-30 19:39
</commit_message>
<xml_diff>
--- a/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
+++ b/Bortoff_Strick_1993/Bortoff_Strick_1993_Table1_snapshot.xlsx
@@ -872,13 +872,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA933C46-8D80-48A1-943D-6FF7CBCBDD2F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA4DC3DE-64B5-4A35-B0E4-424186C53D13}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B3CC3FA-B2EA-4EA2-82F7-4F16E6897E69}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66DDDCDF-0759-497D-8B3D-FE07D27FFF99}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A0BC28A-337D-469B-9D7B-B2ED6855629D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA19CBD5-4048-4F23-A0E9-248656D5D1C7}"/>
 </file>
</xml_diff>